<commit_message>
Keep Excel acceptance markers visibly inside source print areas
</commit_message>
<xml_diff>
--- a/app/src/debug/assets/office-fixtures/workbook-edge.xlsx
+++ b/app/src/debug/assets/office-fixtures/workbook-edge.xlsx
@@ -34,7 +34,7 @@
     <numFmt numFmtId="165" formatCode="dd.mm.yyyy"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +45,10 @@
     <font>
       <name val="Liberation Sans"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Liberation Sans"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="3">
@@ -155,10 +159,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -2583,7 +2593,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
           <t>12-1</t>
@@ -2619,7 +2629,7 @@
           <t>12-7</t>
         </is>
       </c>
-      <c r="H12" s="1" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>ПРАВЫЙ КРАЙ</t>
         </is>
@@ -3765,13 +3775,13 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="24" customHeight="1">
+    <row r="100" ht="30" customHeight="1">
       <c r="A100" t="inlineStr">
         <is>
           <t>СТРОКА-100</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr">
+      <c r="H100" s="3" t="inlineStr">
         <is>
           <t>КОНЕЦ ВЫСОТЫ</t>
         </is>
@@ -4354,7 +4364,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="B2" s="1" t="n"/>
-      <ns0:c r="C2" s="2" t="n">
+      <ns0:c r="C2" s="4" t="n">
         <ns0:v>45351</ns0:v>
       </ns0:c>
       <ns0:c r="D2" s="1" t="n"/>
@@ -4370,7 +4380,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="B3" s="1" t="n"/>
-      <ns0:c r="C3" s="3" t="n">
+      <ns0:c r="C3" s="5" t="n">
         <ns0:v>0.125</ns0:v>
       </ns0:c>
       <ns0:c r="D3" s="1" t="n"/>
@@ -4386,7 +4396,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="B4" s="1" t="n"/>
-      <ns0:c r="C4" s="4" t="n">
+      <ns0:c r="C4" s="6" t="n">
         <ns0:v>-1234.5</ns0:v>
       </ns0:c>
       <ns0:c r="D4" s="1" t="n"/>
@@ -4402,7 +4412,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="B5" s="1" t="n"/>
-      <ns0:c r="C5" s="5" t="n">
+      <ns0:c r="C5" s="7" t="n">
         <ns0:v>125000000</ns0:v>
       </ns0:c>
       <ns0:c r="D5" s="1" t="n"/>
@@ -4418,7 +4428,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="B6" s="1" t="n"/>
-      <ns0:c r="C6" s="6" t="n">
+      <ns0:c r="C6" s="8" t="n">
         <ns0:v>0</ns0:v>
       </ns0:c>
       <ns0:c r="D6" s="1" t="n"/>
@@ -4434,7 +4444,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="B7" s="1" t="n"/>
-      <ns0:c r="C7" s="6" t="n">
+      <ns0:c r="C7" s="8" t="n">
         <ns0:v>1.235</ns0:v>
       </ns0:c>
       <ns0:c r="D7" s="1" t="n"/>
@@ -4450,7 +4460,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="B8" s="1" t="n"/>
-      <ns0:c r="C8" s="6">
+      <ns0:c r="C8" s="8">
         <ns0:f>SUM(10,20,30)</ns0:f>
         <ns0:v>60</ns0:v>
       </ns0:c>
@@ -4467,7 +4477,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="B9" s="1" t="n"/>
-      <ns0:c r="C9" s="6">
+      <ns0:c r="C9" s="8">
         <ns0:f>IF(2&gt;1,42,0)</ns0:f>
         <ns0:v>42</ns0:v>
       </ns0:c>
@@ -4505,28 +4515,28 @@
       <ns0:c r="H11" s="1" t="n"/>
     </ns0:row>
     <ns0:row r="12">
-      <ns0:c r="A12" s="7" t="inlineStr">
+      <ns0:c r="A12" s="9" t="inlineStr">
         <ns0:is>
           <ns0:t>ОБЪЕДИНЕНИЕ И ПЕРЕНОС
 ВТОРАЯ СТРОКА</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="B12" s="8" t="n"/>
-      <ns0:c r="C12" s="8" t="n"/>
-      <ns0:c r="D12" s="9" t="n"/>
+      <ns0:c r="B12" s="10" t="n"/>
+      <ns0:c r="C12" s="10" t="n"/>
+      <ns0:c r="D12" s="11" t="n"/>
       <ns0:c r="E12" s="1" t="n"/>
       <ns0:c r="F12" s="1" t="n"/>
       <ns0:c r="G12" s="1" t="n"/>
       <ns0:c r="H12" s="1" t="n"/>
     </ns0:row>
     <ns0:row r="13">
-      <ns0:c r="A13" s="10" t="n"/>
-      <ns0:c r="B13" s="11" t="n"/>
-      <ns0:c r="C13" s="11" t="n"/>
-      <ns0:c r="D13" s="12" t="n"/>
+      <ns0:c r="A13" s="12" t="n"/>
+      <ns0:c r="B13" s="13" t="n"/>
+      <ns0:c r="C13" s="13" t="n"/>
+      <ns0:c r="D13" s="14" t="n"/>
     </ns0:row>
-    <ns0:row r="14">
-      <ns0:c r="D14" t="inlineStr">
+    <ns0:row r="14" ht="30" customHeight="1">
+      <ns0:c r="D14" s="3" t="inlineStr">
         <ns0:is>
           <ns0:t>КОНЕЦ ЧИСЕЛ</ns0:t>
         </ns0:is>

</xml_diff>